<commit_message>
Berechne Titel und Systemname aus Buchungscode für Touren und Kurse
Titel/Systemname sind mit der Sektion Trier abgesprochen: Titel =
"<Buchungscode> <Formular-Titel>", Systemname = "<Jahr> <Buchungscode>
<Formular-Titel>".
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/touren_tr.xlsx
+++ b/tests/fixtures/expected/touren_tr.xlsx
@@ -621,7 +621,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2606KSKlettersteigtourTraversata</t>
+          <t>26 TR2026-001 Klettersteigtour Traversata</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Klettersteigtour Traversata</t>
+          <t>TR2026-001 Klettersteigtour Traversata</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -738,7 +738,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2605WANFamilienwanderungRuwertal</t>
+          <t>26 TR2026-002 Familienwanderung Ruwertal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Familienwanderung Ruwertal</t>
+          <t>TR2026-002 Familienwanderung Ruwertal</t>
         </is>
       </c>
       <c r="E3" t="n">

</xml_diff>

<commit_message>
Setze bookingState 'wenige frei' bei höchstens 10 maximalen Teilnehmenden
Abgesprochen mit der Sektion Trier: Maßgeblich ist die maximale (nicht die
aktuelle) Teilnehmerzahl aus dem Formular. Gilt für Touren und Kurse; bei mehr
als 10, unbegrenzt oder fehlender Angabe bleibt der Status leer. Ergänzt
anonyme Beispieldaten und Regressionstest für Kurse.
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/touren_tr.xlsx
+++ b/tests/fixtures/expected/touren_tr.xlsx
@@ -704,7 +704,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="n">
+        <v>391</v>
+      </c>
       <c r="AB2" t="inlineStr">
         <is>
           <t>&lt;p&gt;Mitglieder: 15&lt;br /&gt;Die Kosten für Anreise, Unterkunft und Verpflegung muss jeder Teilnehmer selbst tragen. Die Teilnehmer eines außerhalb der Region stattfindenden Ausbildungskurses oder einer Ausbildungstour ermöglichen dem Kursleiter bzw. weiteren Ausbildern eine kostenfreie An- und Abreise. Einzelheiten sind mit dem Kursleiter zu klären.&lt;/p&gt;</t>

</xml_diff>